<commit_message>
Account Payable Step and Line Items Columns Mapping Updated
</commit_message>
<xml_diff>
--- a/src/assets/PO Master.xlsx
+++ b/src/assets/PO Master.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="198">
   <si>
     <t>PO Number</t>
   </si>
@@ -581,15 +581,47 @@
   </si>
   <si>
     <t>PO-31002</t>
+  </si>
+  <si>
+    <t>PO-1045</t>
+  </si>
+  <si>
+    <t>Quantum Office Essentials</t>
+  </si>
+  <si>
+    <t>789 Pine Ave, Calgary, ON</t>
+  </si>
+  <si>
+    <t>100 Business Park Drive</t>
+  </si>
+  <si>
+    <t>2025-07-26</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>6326.87</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>Mouse</t>
+  </si>
+  <si>
+    <t>Headset</t>
+  </si>
+  <si>
+    <t>Laptop</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -643,7 +675,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -671,18 +703,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -964,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
@@ -1500,60 +1530,89 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="29.25">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="C19" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="F19" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="G19" s="14" t="s">
+      <c r="G19" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="H19" s="16">
+      <c r="H19" s="14">
         <v>1582</v>
       </c>
-      <c r="I19" s="14" t="s">
+      <c r="I19" s="13" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="29.25">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="C20" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="E20" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="F20" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="G20" s="14" t="s">
+      <c r="G20" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="H20" s="16">
+      <c r="H20" s="14">
         <v>1582</v>
       </c>
-      <c r="I20" s="14" t="s">
+      <c r="I20" s="13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="H21" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="I21" s="15" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1564,7 +1623,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.85546875" style="1" customWidth="1"/>
@@ -2308,10 +2367,10 @@
       <c r="H18" s="10">
         <v>6</v>
       </c>
-      <c r="I18" s="13">
+      <c r="I18" s="11">
         <v>254</v>
       </c>
-      <c r="J18" s="13">
+      <c r="J18" s="11">
         <v>1524</v>
       </c>
       <c r="K18" s="10" t="s">
@@ -2349,10 +2408,10 @@
       <c r="H19" s="10">
         <v>9</v>
       </c>
-      <c r="I19" s="13">
+      <c r="I19" s="11">
         <v>270</v>
       </c>
-      <c r="J19" s="13">
+      <c r="J19" s="11">
         <v>2430</v>
       </c>
       <c r="K19" s="10" t="s">
@@ -2390,10 +2449,10 @@
       <c r="H20" s="10">
         <v>3</v>
       </c>
-      <c r="I20" s="13">
+      <c r="I20" s="11">
         <v>217</v>
       </c>
-      <c r="J20" s="13">
+      <c r="J20" s="11">
         <v>651</v>
       </c>
       <c r="K20" s="10" t="s">
@@ -2431,10 +2490,10 @@
       <c r="H21" s="10">
         <v>6</v>
       </c>
-      <c r="I21" s="13">
+      <c r="I21" s="11">
         <v>254</v>
       </c>
-      <c r="J21" s="13">
+      <c r="J21" s="11">
         <v>1524</v>
       </c>
       <c r="K21" s="10" t="s">
@@ -2472,10 +2531,10 @@
       <c r="H22" s="10">
         <v>9</v>
       </c>
-      <c r="I22" s="13">
+      <c r="I22" s="11">
         <v>270</v>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="11">
         <v>2430</v>
       </c>
       <c r="K22" s="10" t="s">
@@ -2513,10 +2572,10 @@
       <c r="H23" s="10">
         <v>3</v>
       </c>
-      <c r="I23" s="13">
+      <c r="I23" s="11">
         <v>217</v>
       </c>
-      <c r="J23" s="13">
+      <c r="J23" s="11">
         <v>651</v>
       </c>
       <c r="K23" s="10" t="s">
@@ -2554,10 +2613,10 @@
       <c r="H24" s="10">
         <v>6</v>
       </c>
-      <c r="I24" s="13">
+      <c r="I24" s="11">
         <v>254</v>
       </c>
-      <c r="J24" s="13">
+      <c r="J24" s="11">
         <v>1524</v>
       </c>
       <c r="K24" s="10" t="s">
@@ -2595,10 +2654,10 @@
       <c r="H25" s="10">
         <v>9</v>
       </c>
-      <c r="I25" s="13">
+      <c r="I25" s="11">
         <v>270</v>
       </c>
-      <c r="J25" s="13">
+      <c r="J25" s="11">
         <v>2430</v>
       </c>
       <c r="K25" s="10" t="s">
@@ -2636,10 +2695,10 @@
       <c r="H26" s="10">
         <v>3</v>
       </c>
-      <c r="I26" s="13">
+      <c r="I26" s="11">
         <v>217</v>
       </c>
-      <c r="J26" s="13">
+      <c r="J26" s="11">
         <v>651</v>
       </c>
       <c r="K26" s="10" t="s">
@@ -2677,10 +2736,10 @@
       <c r="H27" s="10">
         <v>6</v>
       </c>
-      <c r="I27" s="13">
+      <c r="I27" s="11">
         <v>254</v>
       </c>
-      <c r="J27" s="13">
+      <c r="J27" s="11">
         <v>1524</v>
       </c>
       <c r="K27" s="10" t="s">
@@ -2718,10 +2777,10 @@
       <c r="H28" s="10">
         <v>9</v>
       </c>
-      <c r="I28" s="13">
+      <c r="I28" s="11">
         <v>270</v>
       </c>
-      <c r="J28" s="13">
+      <c r="J28" s="11">
         <v>2430</v>
       </c>
       <c r="K28" s="10" t="s">
@@ -2759,10 +2818,10 @@
       <c r="H29" s="10">
         <v>3</v>
       </c>
-      <c r="I29" s="13">
+      <c r="I29" s="11">
         <v>217</v>
       </c>
-      <c r="J29" s="13">
+      <c r="J29" s="11">
         <v>651</v>
       </c>
       <c r="K29" s="10" t="s">
@@ -2800,10 +2859,10 @@
       <c r="H30" s="10">
         <v>6</v>
       </c>
-      <c r="I30" s="13">
+      <c r="I30" s="11">
         <v>254</v>
       </c>
-      <c r="J30" s="13">
+      <c r="J30" s="11">
         <v>1524</v>
       </c>
       <c r="K30" s="10" t="s">
@@ -2841,10 +2900,10 @@
       <c r="H31" s="10">
         <v>9</v>
       </c>
-      <c r="I31" s="13">
+      <c r="I31" s="11">
         <v>270</v>
       </c>
-      <c r="J31" s="13">
+      <c r="J31" s="11">
         <v>2430</v>
       </c>
       <c r="K31" s="10" t="s">
@@ -2882,10 +2941,10 @@
       <c r="H32" s="10">
         <v>3</v>
       </c>
-      <c r="I32" s="13">
+      <c r="I32" s="11">
         <v>217</v>
       </c>
-      <c r="J32" s="13">
+      <c r="J32" s="11">
         <v>651</v>
       </c>
       <c r="K32" s="10" t="s">
@@ -3145,170 +3204,241 @@
       </c>
     </row>
     <row r="39" spans="1:13" ht="43.5">
-      <c r="A39" s="14" t="s">
+      <c r="A39" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="B39" s="14">
+      <c r="B39" s="13">
         <v>1</v>
       </c>
-      <c r="C39" s="14" t="s">
+      <c r="C39" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="D39" s="14" t="s">
+      <c r="D39" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E39" s="14" t="s">
+      <c r="E39" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="F39" s="14" t="s">
+      <c r="F39" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="G39" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="H39" s="14">
+      <c r="G39" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="H39" s="13">
         <v>2</v>
       </c>
-      <c r="I39" s="15">
+      <c r="I39" s="14">
         <v>250</v>
       </c>
-      <c r="J39" s="15">
+      <c r="J39" s="14">
         <v>500</v>
       </c>
-      <c r="K39" s="14" t="s">
+      <c r="K39" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L39" s="14" t="s">
+      <c r="L39" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="M39" s="14" t="s">
+      <c r="M39" s="13" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="43.5">
-      <c r="A40" s="14" t="s">
+      <c r="A40" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="B40" s="14">
+      <c r="B40" s="13">
         <v>2</v>
       </c>
-      <c r="C40" s="14" t="s">
+      <c r="C40" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="D40" s="14" t="s">
+      <c r="D40" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E40" s="14" t="s">
+      <c r="E40" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="F40" s="14" t="s">
+      <c r="F40" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="G40" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="H40" s="14">
+      <c r="G40" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="H40" s="13">
         <v>3</v>
       </c>
-      <c r="I40" s="15">
+      <c r="I40" s="14">
         <v>300</v>
       </c>
-      <c r="J40" s="15">
+      <c r="J40" s="14">
         <v>900</v>
       </c>
-      <c r="K40" s="14" t="s">
+      <c r="K40" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L40" s="14" t="s">
+      <c r="L40" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="M40" s="14" t="s">
+      <c r="M40" s="13" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="41" spans="1:13" ht="43.5">
-      <c r="A41" s="14" t="s">
+      <c r="A41" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="B41" s="14">
+      <c r="B41" s="13">
         <v>1</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="C41" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="D41" s="14" t="s">
+      <c r="D41" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E41" s="14" t="s">
+      <c r="E41" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="F41" s="14" t="s">
+      <c r="F41" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="G41" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="H41" s="14">
+      <c r="G41" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="H41" s="13">
         <v>2</v>
       </c>
-      <c r="I41" s="15">
+      <c r="I41" s="14">
         <v>250</v>
       </c>
-      <c r="J41" s="15">
+      <c r="J41" s="14">
         <v>500</v>
       </c>
-      <c r="K41" s="14" t="s">
+      <c r="K41" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L41" s="14" t="s">
+      <c r="L41" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="M41" s="14" t="s">
+      <c r="M41" s="13" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="43.5">
-      <c r="A42" s="14" t="s">
+      <c r="A42" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="B42" s="14">
+      <c r="B42" s="13">
         <v>2</v>
       </c>
-      <c r="C42" s="14" t="s">
+      <c r="C42" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="D42" s="14" t="s">
+      <c r="D42" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E42" s="14" t="s">
+      <c r="E42" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="F42" s="14" t="s">
+      <c r="F42" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="G42" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="H42" s="14">
+      <c r="G42" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="H42" s="13">
         <v>3</v>
       </c>
-      <c r="I42" s="15">
+      <c r="I42" s="14">
         <v>300</v>
       </c>
-      <c r="J42" s="15">
+      <c r="J42" s="14">
         <v>900</v>
       </c>
-      <c r="K42" s="14" t="s">
+      <c r="K42" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="L42" s="14" t="s">
+      <c r="L42" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="M42" s="14" t="s">
+      <c r="M42" s="13" t="s">
         <v>150</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="E43" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="H43" s="18">
+        <v>9</v>
+      </c>
+      <c r="I43" s="9">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13">
+      <c r="A44" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="E44" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="H44" s="18">
+        <v>1</v>
+      </c>
+      <c r="I44" s="9">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13">
+      <c r="A45" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="E45" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="H45" s="18">
+        <v>6</v>
+      </c>
+      <c r="I45" s="9">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13">
+      <c r="A46" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="E46" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="H46" s="18">
+        <v>6</v>
+      </c>
+      <c r="I46" s="9">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13">
+      <c r="A47" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="E47" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="H47" s="18">
+        <v>2</v>
+      </c>
+      <c r="I47" s="9">
+        <v>84</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>